<commit_message>
Registro BUG-01 validacion de busqueda vacia
</commit_message>
<xml_diff>
--- a/bugs/reporte_bugs.xlsx
+++ b/bugs/reporte_bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\bugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713A30B3-378A-4795-8D62-C81C8AE6FA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05DB729E-35EA-4658-B7B6-AC44E2D6B289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BE1C2E9C-754A-4331-9015-9AE0A4AB5D3F}"/>
   </bookViews>
@@ -36,13 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>BUG-ID</t>
-  </si>
-  <si>
-    <t>Descripcion</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Precondiciones</t>
   </si>
@@ -50,26 +44,101 @@
     <t>Pasos</t>
   </si>
   <si>
-    <t>Resultados esperados</t>
-  </si>
-  <si>
     <t>Resultado obtenido</t>
   </si>
   <si>
-    <t>Prioridad/severidad</t>
+    <t>BUG-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categoria </t>
+  </si>
+  <si>
+    <t>Resultado esperado</t>
+  </si>
+  <si>
+    <t>Prioridad</t>
+  </si>
+  <si>
+    <t>Severidad</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>Búsqueda</t>
+  </si>
+  <si>
+    <t>Bug-ID</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Ejecutar búsqueda sin longin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usar Chrome en Windows. </t>
+  </si>
+  <si>
+    <t>1.Ir a Pinterest web.
+2.Hacer clic en barra de búsqueda.
+3.Dejar el campo vacío.
+4.Presionar Enter.</t>
+  </si>
+  <si>
+    <t>El sistema debería mostrar mensaje indicando que debe ingresar un término de búsqueda o evitar ejecutar la acción.</t>
+  </si>
+  <si>
+    <t>No se muestra mensaje ni acción alguna; el sistema no responde visualmente.</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>Fail</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos "/>
     </font>
   </fonts>
   <fills count="2">
@@ -92,8 +161,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -428,37 +507,257 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75AFE187-FC29-4EA5-B4B4-407E3DADF7F0}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" customWidth="1"/>
     <col min="5" max="5" width="22.85546875" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="26.5703125" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" ht="18.75">
+      <c r="A1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="75">
+      <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
+      <c r="B2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Agrego evidencia BUG-01 busqueda vacia
</commit_message>
<xml_diff>
--- a/bugs/reporte_bugs.xlsx
+++ b/bugs/reporte_bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\bugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05DB729E-35EA-4658-B7B6-AC44E2D6B289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C346479C-D388-48A0-99A7-D4672448C488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BE1C2E9C-754A-4331-9015-9AE0A4AB5D3F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Precondiciones</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t>Estado</t>
-  </si>
-  <si>
-    <t>Observaciones</t>
   </si>
   <si>
     <t>Búsqueda</t>
@@ -102,6 +99,12 @@
   </si>
   <si>
     <t>Fail</t>
+  </si>
+  <si>
+    <t>Evidencias</t>
+  </si>
+  <si>
+    <t>BUG-01_busqueda_vacia_sin_validacion.png</t>
   </si>
 </sst>
 </file>
@@ -524,13 +527,13 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.75">
       <c r="A1" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -554,7 +557,7 @@
         <v>8</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="75">
@@ -562,33 +565,35 @@
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="4"/>
+      <c r="K2" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="4"/>

</xml_diff>

<commit_message>
Registro BUG-02 busqueda con caracteres especiales
</commit_message>
<xml_diff>
--- a/bugs/reporte_bugs.xlsx
+++ b/bugs/reporte_bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\bugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C346479C-D388-48A0-99A7-D4672448C488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74E0E7F8-0B5B-48D9-BAD0-6A82D10DEE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BE1C2E9C-754A-4331-9015-9AE0A4AB5D3F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>Precondiciones</t>
   </si>
@@ -105,13 +105,52 @@
   </si>
   <si>
     <t>BUG-01_busqueda_vacia_sin_validacion.png</t>
+  </si>
+  <si>
+    <t>BUG-02</t>
+  </si>
+  <si>
+    <t>Búsqueda con caracteres especiales devuelve resultados irrelevantes sin advertencia</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Utilizar los caracteres </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>@#$%</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Abrir Pinterest web sin iniciar sesión.
+2.En la barra de búsqueda escribir @#$%.
+3.Presionar Enter.</t>
+  </si>
+  <si>
+    <t>El sistema debería:
+-Mostrar mensaje “término inválido” o
+-Mostrar “sin resultados” o
+-Ignorar símbolos y buscar por contenido relacionado (con algún feedback).</t>
+  </si>
+  <si>
+    <t>Muestra resultados variados no relacionados (ej. gatos/corazones) sin advertencia ni mensaje.</t>
+  </si>
+  <si>
+    <t>BUG-02_busqueda_caracteres_especiales_resultados_irrelevantes.png</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,6 +181,14 @@
       <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos "/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -595,18 +642,36 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="4"/>
+    <row r="3" spans="1:11" ht="105">
+      <c r="A3" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+      <c r="C3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
+      <c r="K3" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="4"/>

</xml_diff>

<commit_message>
Agrego evidencia adicional a BUG-02 termino inexistente
</commit_message>
<xml_diff>
--- a/bugs/reporte_bugs.xlsx
+++ b/bugs/reporte_bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\bugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74E0E7F8-0B5B-48D9-BAD0-6A82D10DEE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3310CF-DEE7-42FC-864B-647400717A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BE1C2E9C-754A-4331-9015-9AE0A4AB5D3F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>Precondiciones</t>
   </si>
@@ -143,7 +143,13 @@
     <t>Muestra resultados variados no relacionados (ej. gatos/corazones) sin advertencia ni mensaje.</t>
   </si>
   <si>
-    <t>BUG-02_busqueda_caracteres_especiales_resultados_irrelevantes.png</t>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>También ocurre cuando se ingresa un término inexistente, mostrando resultados no relacionados sin mensaje de “sin resultados” o sugerencias.</t>
+  </si>
+  <si>
+    <t>BUG-02_busqueda_caracteres_especiales_resultados_irrelevantes.png                                     BUG-02_busqueda_termino_inexistente_resultados_irrelevantes.png</t>
   </si>
 </sst>
 </file>
@@ -557,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75AFE187-FC29-4EA5-B4B4-407E3DADF7F0}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
@@ -570,9 +576,10 @@
     <col min="8" max="8" width="15.28515625" customWidth="1"/>
     <col min="9" max="9" width="16.5703125" customWidth="1"/>
     <col min="11" max="11" width="18.7109375" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75">
+    <row r="1" spans="1:12" ht="18.75">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -606,8 +613,11 @@
       <c r="K1" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="75">
+      <c r="L1" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="75">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -642,7 +652,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="105">
+    <row r="3" spans="1:12" ht="150">
       <c r="A3" s="4" t="s">
         <v>22</v>
       </c>
@@ -670,10 +680,13 @@
       </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>30</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -686,7 +699,7 @@
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -699,7 +712,7 @@
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -712,7 +725,7 @@
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -725,7 +738,7 @@
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -738,7 +751,7 @@
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -751,7 +764,7 @@
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:12">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -764,7 +777,7 @@
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:12">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -777,7 +790,7 @@
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:12">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -790,7 +803,7 @@
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:12">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -803,7 +816,7 @@
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:12">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -816,7 +829,7 @@
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:12">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>

</xml_diff>

<commit_message>
Registro BUG-03 enlace externo del pin con error
</commit_message>
<xml_diff>
--- a/bugs/reporte_bugs.xlsx
+++ b/bugs/reporte_bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\bugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3310CF-DEE7-42FC-864B-647400717A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB61150-1F54-4E9E-8FD3-7924CC4CA074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BE1C2E9C-754A-4331-9015-9AE0A4AB5D3F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>Precondiciones</t>
   </si>
@@ -96,9 +96,6 @@
   </si>
   <si>
     <t>Baja</t>
-  </si>
-  <si>
-    <t>Fail</t>
   </si>
   <si>
     <t>Evidencias</t>
@@ -151,12 +148,45 @@
   <si>
     <t>BUG-02_busqueda_caracteres_especiales_resultados_irrelevantes.png                                     BUG-02_busqueda_termino_inexistente_resultados_irrelevantes.png</t>
   </si>
+  <si>
+    <t>BUG-03_enlace_externo_error_xml.png</t>
+  </si>
+  <si>
+    <t>BUG-03</t>
+  </si>
+  <si>
+    <t>Enlace “Visitar” redirige a página con error XML (sitio externo)</t>
+  </si>
+  <si>
+    <t>Detalle del pin</t>
+  </si>
+  <si>
+    <t>1.Abrir Pinterest web.
+2.Abrir un pin (ej. imagen de uña).
+3.Clic en “Visitar” / enlace externo.
+4.Observar la página destino en la nueva pestaña.</t>
+  </si>
+  <si>
+    <t>Seleccionar un pin.</t>
+  </si>
+  <si>
+    <t>El enlace externo debería abrir el sitio destino con contenido disponible.</t>
+  </si>
+  <si>
+    <t>Se abre una nueva pestaña pero muestra una página de error XML (UserProjectAccountProblem / billing account closed).</t>
+  </si>
+  <si>
+    <t>Nuevo</t>
+  </si>
+  <si>
+    <t>URL DEL SITIO DESTINO https://storage.googleapis.com/daegu2484/pin-on-uniqqogifts-2E6C3B.jpg?utm_source=Pinterest&amp;utm_medium=organic</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -196,6 +226,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -214,10 +252,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -229,8 +268,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -611,10 +654,10 @@
         <v>8</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="75">
@@ -646,31 +689,31 @@
         <v>18</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="150">
       <c r="A3" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>18</v>
@@ -678,26 +721,53 @@
       <c r="I3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="4"/>
+      <c r="J3" s="4" t="s">
+        <v>38</v>
+      </c>
       <c r="K3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="120">
+      <c r="A4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
+      <c r="L4" s="5" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="4"/>
@@ -843,6 +913,9 @@
       <c r="K15" s="4"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="L4" r:id="rId1" display="https://storage.googleapis.com/daegu2484/pin-on-uniqqogifts-2E6C3B.jpg?utm_source=Pinterest&amp;utm_medium=organic" xr:uid="{B3B974F3-A0CD-41AB-BB5E-6684081752D3}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualice matriz y reporte de bugs con detalles finales
</commit_message>
<xml_diff>
--- a/bugs/reporte_bugs.xlsx
+++ b/bugs/reporte_bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\bugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB61150-1F54-4E9E-8FD3-7924CC4CA074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBB321A2-6D26-49DE-96E3-D5587BB37640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BE1C2E9C-754A-4331-9015-9AE0A4AB5D3F}"/>
   </bookViews>
@@ -107,9 +107,6 @@
     <t>BUG-02</t>
   </si>
   <si>
-    <t>Búsqueda con caracteres especiales devuelve resultados irrelevantes sin advertencia</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Utilizar los caracteres </t>
     </r>
@@ -155,9 +152,6 @@
     <t>BUG-03</t>
   </si>
   <si>
-    <t>Enlace “Visitar” redirige a página con error XML (sitio externo)</t>
-  </si>
-  <si>
     <t>Detalle del pin</t>
   </si>
   <si>
@@ -180,6 +174,12 @@
   </si>
   <si>
     <t>URL DEL SITIO DESTINO https://storage.googleapis.com/daegu2484/pin-on-uniqqogifts-2E6C3B.jpg?utm_source=Pinterest&amp;utm_medium=organic</t>
+  </si>
+  <si>
+    <t>Búsqueda con caracteres especiales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visitar el enlace que proporciona el pin. </t>
   </si>
 </sst>
 </file>
@@ -657,7 +657,7 @@
         <v>19</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="75">
@@ -689,7 +689,7 @@
         <v>18</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>20</v>
@@ -701,19 +701,19 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>18</v>
@@ -722,36 +722,36 @@
         <v>17</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="120">
       <c r="A4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="F4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>37</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>17</v>
@@ -760,13 +760,13 @@
         <v>17</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:12">

</xml_diff>